<commit_message>
Write test cases for login page
</commit_message>
<xml_diff>
--- a/testCases/testCases.xlsx
+++ b/testCases/testCases.xlsx
@@ -1,13 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\projects\paraBank\testCases\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED0AF95-65EC-48D7-B5A5-05E9B427121E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="User Registration" sheetId="2" r:id="rId2"/>
+    <sheet name="Open New Account" sheetId="3" r:id="rId3"/>
+    <sheet name="Accounts Overview" sheetId="4" r:id="rId4"/>
+    <sheet name="Transfer Funds" sheetId="5" r:id="rId5"/>
+    <sheet name="Bill Payment" sheetId="6" r:id="rId6"/>
+    <sheet name="Find Transactions" sheetId="7" r:id="rId7"/>
+    <sheet name="Update Contact Information" sheetId="8" r:id="rId8"/>
+    <sheet name="Request Loan" sheetId="9" r:id="rId9"/>
+    <sheet name="LogOut &amp; Session Management" sheetId="10" r:id="rId10"/>
+    <sheet name="UI &amp; Navigation Testing" sheetId="11" r:id="rId11"/>
+    <sheet name="Security" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,12 +35,287 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="81">
+  <si>
+    <t>Test ID</t>
+  </si>
+  <si>
+    <t>Test Scenario</t>
+  </si>
+  <si>
+    <t>Test case</t>
+  </si>
+  <si>
+    <t>Precondition</t>
+  </si>
+  <si>
+    <t>Test data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected resutl </t>
+  </si>
+  <si>
+    <t>Actual result</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>TC_001</t>
+  </si>
+  <si>
+    <t>Verify Login with valid credentials</t>
+  </si>
+  <si>
+    <t>Check login with valid username &amp; password</t>
+  </si>
+  <si>
+    <t>Mustbe register User</t>
+  </si>
+  <si>
+    <t>Valid credentials</t>
+  </si>
+  <si>
+    <t>User successfully login</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Criticale</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>TC_006</t>
+  </si>
+  <si>
+    <t>TC_007</t>
+  </si>
+  <si>
+    <t>TC_008</t>
+  </si>
+  <si>
+    <t>TC_009</t>
+  </si>
+  <si>
+    <t>TC_010</t>
+  </si>
+  <si>
+    <t>TC_011</t>
+  </si>
+  <si>
+    <t>TC_012</t>
+  </si>
+  <si>
+    <t>TC_013</t>
+  </si>
+  <si>
+    <t>Verify Login with invalid credentials</t>
+  </si>
+  <si>
+    <t>Check login with invalid username &amp; password</t>
+  </si>
+  <si>
+    <t>Login page open</t>
+  </si>
+  <si>
+    <t>Invalid credentials</t>
+  </si>
+  <si>
+    <t>User not login &amp; an error
+message show.</t>
+  </si>
+  <si>
+    <t>major</t>
+  </si>
+  <si>
+    <t>Verify Login with Invalid password</t>
+  </si>
+  <si>
+    <t>Check login with invalid password</t>
+  </si>
+  <si>
+    <t>Invalid password</t>
+  </si>
+  <si>
+    <t>Verify Login with Invalid username</t>
+  </si>
+  <si>
+    <t>Check login with invalid username</t>
+  </si>
+  <si>
+    <t>Invalid username</t>
+  </si>
+  <si>
+    <t>Verify both field empty</t>
+  </si>
+  <si>
+    <t>Check login with empty field</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Check with valid username &amp; empty password</t>
+  </si>
+  <si>
+    <t>valid username &amp;
+empty password</t>
+  </si>
+  <si>
+    <t>Verify with empty username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify with empty password </t>
+  </si>
+  <si>
+    <t>Check with empty username &amp; valid password</t>
+  </si>
+  <si>
+    <t>empty username &amp; 
+valid password</t>
+  </si>
+  <si>
+    <t>Verify with leading spaces username</t>
+  </si>
+  <si>
+    <t>Check with leading spaces username</t>
+  </si>
+  <si>
+    <t>leading spaces with
+username &amp; valid
+password</t>
+  </si>
+  <si>
+    <t>Application handles 
+whitespace consistently</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Minor</t>
+  </si>
+  <si>
+    <t>Verify with password case sensitivity</t>
+  </si>
+  <si>
+    <t>Check password case sensitivity</t>
+  </si>
+  <si>
+    <t>Registred user</t>
+  </si>
+  <si>
+    <t>Incorrect password</t>
+  </si>
+  <si>
+    <t>Major</t>
+  </si>
+  <si>
+    <t>passed</t>
+  </si>
+  <si>
+    <t>Verify username with special 
+character</t>
+  </si>
+  <si>
+    <t>Check useranem with special character</t>
+  </si>
+  <si>
+    <t>()&amp;(*&amp;^</t>
+  </si>
+  <si>
+    <t>Input handle safely</t>
+  </si>
+  <si>
+    <t>Verify password masking</t>
+  </si>
+  <si>
+    <t>Check password is masking</t>
+  </si>
+  <si>
+    <t>password1234</t>
+  </si>
+  <si>
+    <t>password should be masked</t>
+  </si>
+  <si>
+    <t>password masked</t>
+  </si>
+  <si>
+    <t>Verify forgot password</t>
+  </si>
+  <si>
+    <t>Check forgot password</t>
+  </si>
+  <si>
+    <t>Navigate to password recovery page</t>
+  </si>
+  <si>
+    <t>Hight</t>
+  </si>
+  <si>
+    <t>Verify login after logout</t>
+  </si>
+  <si>
+    <t>Check login after logout</t>
+  </si>
+  <si>
+    <t>User loged in</t>
+  </si>
+  <si>
+    <t>User should not remain 
+authenticated unexpectedly</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -49,8 +341,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,7 +635,640 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B5:K25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="2:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" s="3" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K15" s="3"/>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="63" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12163991-9993-46BC-8960-6F56B743FC05}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BAE5816-1012-42FF-971C-CD7A330BA13D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DF8A9D9-635E-445B-9177-811C872929E6}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA7331C2-AA49-4852-97B7-FA6B421ADFE5}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE974E59-5E92-4F37-80CF-F5CD1890B612}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7368FBBA-23E1-4E37-B79D-DA8AF23D4CC8}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4522ED92-A484-468F-A273-7D2FF8FE5E89}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E020456B-E449-436C-B4A1-83C24244656B}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A65531-C65D-4E87-93C4-F541C3027ABE}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E373737-E2CF-4C9B-84C2-B39504254411}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08542F11-BF3E-45D3-83AB-946027AB8110}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>

<commit_message>
Write registration test cases for para bank
</commit_message>
<xml_diff>
--- a/testCases/testCases.xlsx
+++ b/testCases/testCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\projects\paraBank\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED0AF95-65EC-48D7-B5A5-05E9B427121E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6661752-0925-4DFB-997C-7B1BB31B4FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="124">
   <si>
     <t>Test ID</t>
   </si>
@@ -287,6 +287,137 @@
   <si>
     <t>User should not remain 
 authenticated unexpectedly</t>
+  </si>
+  <si>
+    <t>Verify registration with valid information</t>
+  </si>
+  <si>
+    <t>Check registration with valid information</t>
+  </si>
+  <si>
+    <t>Registration page open</t>
+  </si>
+  <si>
+    <t>Valid information</t>
+  </si>
+  <si>
+    <t>Account create successfully</t>
+  </si>
+  <si>
+    <t>Verify with firstname empty</t>
+  </si>
+  <si>
+    <t>first name empty</t>
+  </si>
+  <si>
+    <t>Validation displayed</t>
+  </si>
+  <si>
+    <t>Verify with lastname empty</t>
+  </si>
+  <si>
+    <t>last name empty</t>
+  </si>
+  <si>
+    <t>Verify with address empty</t>
+  </si>
+  <si>
+    <t>address empty</t>
+  </si>
+  <si>
+    <t>Verify with city empty</t>
+  </si>
+  <si>
+    <t>Check with city empty</t>
+  </si>
+  <si>
+    <t>Check with firstname empty</t>
+  </si>
+  <si>
+    <t>Check with lastname empty</t>
+  </si>
+  <si>
+    <t>Verify with state empty</t>
+  </si>
+  <si>
+    <t>Check with state empty</t>
+  </si>
+  <si>
+    <t>Verify with zip code empty</t>
+  </si>
+  <si>
+    <t>check with zip empty</t>
+  </si>
+  <si>
+    <t>Verify with phone empty</t>
+  </si>
+  <si>
+    <t>Verify with username empty</t>
+  </si>
+  <si>
+    <t>Check with username empty</t>
+  </si>
+  <si>
+    <t>Verify with password empty</t>
+  </si>
+  <si>
+    <t>Check with password empty</t>
+  </si>
+  <si>
+    <t>Verify with Confirm password mismatch</t>
+  </si>
+  <si>
+    <t>Check password mismatch</t>
+  </si>
+  <si>
+    <t>City empty</t>
+  </si>
+  <si>
+    <t>state empty</t>
+  </si>
+  <si>
+    <t>zip code empty</t>
+  </si>
+  <si>
+    <t>phone emtpy</t>
+  </si>
+  <si>
+    <t>username empty</t>
+  </si>
+  <si>
+    <t>password empty</t>
+  </si>
+  <si>
+    <t>Enter different 
+pasword</t>
+  </si>
+  <si>
+    <t>Verify with duplicate username</t>
+  </si>
+  <si>
+    <t>Check with duplicate password</t>
+  </si>
+  <si>
+    <t>Password mismatch error 
+message display.</t>
+  </si>
+  <si>
+    <t>Existing username</t>
+  </si>
+  <si>
+    <t>registration rejected</t>
+  </si>
+  <si>
+    <t>Verify with very logn input</t>
+  </si>
+  <si>
+    <t>Check registration with long input</t>
+  </si>
+  <si>
+    <t>Enter oversized value</t>
+  </si>
+  <si>
+    <t>Application handels input</t>
   </si>
 </sst>
 </file>
@@ -341,7 +472,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -355,6 +486,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1206,9 +1340,455 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA7331C2-AA49-4852-97B7-FA6B421ADFE5}">
-  <dimension ref="A1"/>
+  <dimension ref="B4:K17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="25.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:11" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H5" t="s">
+        <v>85</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" t="s">
+        <v>88</v>
+      </c>
+      <c r="H6" t="s">
+        <v>88</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" t="s">
+        <v>83</v>
+      </c>
+      <c r="F7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" t="s">
+        <v>88</v>
+      </c>
+      <c r="H7" t="s">
+        <v>88</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D8" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H8" t="s">
+        <v>88</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G9" t="s">
+        <v>88</v>
+      </c>
+      <c r="H9" t="s">
+        <v>88</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" t="s">
+        <v>16</v>
+      </c>
+      <c r="K9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F10" t="s">
+        <v>109</v>
+      </c>
+      <c r="G10" t="s">
+        <v>88</v>
+      </c>
+      <c r="H10" t="s">
+        <v>88</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" t="s">
+        <v>16</v>
+      </c>
+      <c r="K10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G11" t="s">
+        <v>88</v>
+      </c>
+      <c r="H11" t="s">
+        <v>88</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" t="s">
+        <v>111</v>
+      </c>
+      <c r="G12" t="s">
+        <v>88</v>
+      </c>
+      <c r="H12" t="s">
+        <v>88</v>
+      </c>
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E13" t="s">
+        <v>83</v>
+      </c>
+      <c r="F13" t="s">
+        <v>112</v>
+      </c>
+      <c r="G13" t="s">
+        <v>88</v>
+      </c>
+      <c r="H13" t="s">
+        <v>88</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" t="s">
+        <v>16</v>
+      </c>
+      <c r="K13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>104</v>
+      </c>
+      <c r="D14" t="s">
+        <v>105</v>
+      </c>
+      <c r="E14" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" t="s">
+        <v>113</v>
+      </c>
+      <c r="G14" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" t="s">
+        <v>88</v>
+      </c>
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" t="s">
+        <v>107</v>
+      </c>
+      <c r="E15" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+      <c r="J15" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" t="s">
+        <v>116</v>
+      </c>
+      <c r="E16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" t="s">
+        <v>118</v>
+      </c>
+      <c r="G16" t="s">
+        <v>119</v>
+      </c>
+      <c r="H16" t="s">
+        <v>119</v>
+      </c>
+      <c r="I16" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" t="s">
+        <v>16</v>
+      </c>
+      <c r="K16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" t="s">
+        <v>121</v>
+      </c>
+      <c r="E17" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" t="s">
+        <v>122</v>
+      </c>
+      <c r="G17" t="s">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Write test case for open new account
</commit_message>
<xml_diff>
--- a/testCases/testCases.xlsx
+++ b/testCases/testCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\projects\paraBank\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6661752-0925-4DFB-997C-7B1BB31B4FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE26BFD-33AF-44FB-8500-DDED8988FEE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="163">
   <si>
     <t>Test ID</t>
   </si>
@@ -418,6 +418,130 @@
   </si>
   <si>
     <t>Application handels input</t>
+  </si>
+  <si>
+    <t>Verify Open New Account page</t>
+  </si>
+  <si>
+    <t>Logged in</t>
+  </si>
+  <si>
+    <t>Check open new account page</t>
+  </si>
+  <si>
+    <t>Page open</t>
+  </si>
+  <si>
+    <t>Verify create checking account</t>
+  </si>
+  <si>
+    <t>Check create new account</t>
+  </si>
+  <si>
+    <t>Logged in with eligible acount</t>
+  </si>
+  <si>
+    <t>New account created</t>
+  </si>
+  <si>
+    <t>Verify with create saving accounts</t>
+  </si>
+  <si>
+    <t>Check new saving accounts</t>
+  </si>
+  <si>
+    <t>New saving account created</t>
+  </si>
+  <si>
+    <t>New saving account
+ created</t>
+  </si>
+  <si>
+    <t>Verify funding account list</t>
+  </si>
+  <si>
+    <t>Check funding account list</t>
+  </si>
+  <si>
+    <t>Eligible accounts displayed</t>
+  </si>
+  <si>
+    <t>Verify create valid funding account</t>
+  </si>
+  <si>
+    <t>Check create account with 
+valid funding account.</t>
+  </si>
+  <si>
+    <t>Valid account</t>
+  </si>
+  <si>
+    <t>Account created successfully</t>
+  </si>
+  <si>
+    <t>Verify generated account number</t>
+  </si>
+  <si>
+    <t>Check generated account
+number</t>
+  </si>
+  <si>
+    <t>Account created</t>
+  </si>
+  <si>
+    <t>Unique account number display</t>
+  </si>
+  <si>
+    <t>Verify new account in overview</t>
+  </si>
+  <si>
+    <t>Check new account in overview</t>
+  </si>
+  <si>
+    <t>New account appears</t>
+  </si>
+  <si>
+    <t>Verify repeated account</t>
+  </si>
+  <si>
+    <t>Check create repeated account</t>
+  </si>
+  <si>
+    <t>logged in</t>
+  </si>
+  <si>
+    <t>Multiple request</t>
+  </si>
+  <si>
+    <t>Each valid request handle correctly</t>
+  </si>
+  <si>
+    <t>Verify Invalid account / funding 
+selection</t>
+  </si>
+  <si>
+    <t>Check invalid account / funding .
+Selection</t>
+  </si>
+  <si>
+    <t>Attempt invalid
+selection</t>
+  </si>
+  <si>
+    <t>Request rejected safely</t>
+  </si>
+  <si>
+    <t>Verify Rapid multiple submissions</t>
+  </si>
+  <si>
+    <t>Check multiple submissions</t>
+  </si>
+  <si>
+    <t>Click created repeatedly</t>
+  </si>
+  <si>
+    <t>Duplicate unintednded account are 
+not created.</t>
   </si>
 </sst>
 </file>
@@ -472,7 +596,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -489,6 +613,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1795,9 +1925,311 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE974E59-5E92-4F37-80CF-F5CD1890B612}">
-  <dimension ref="A1"/>
+  <dimension ref="A4:K14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" customWidth="1"/>
+    <col min="6" max="6" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="32.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+    </row>
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+    </row>
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="B7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+    </row>
+    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+    </row>
+    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="B10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+    </row>
+    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="B13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+    </row>
+    <row r="14" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="B14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write test cases for account overview
</commit_message>
<xml_diff>
--- a/testCases/testCases.xlsx
+++ b/testCases/testCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\projects\paraBank\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE26BFD-33AF-44FB-8500-DDED8988FEE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47EE7D95-E7F7-4F35-8F25-E6A9E67C8EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="192">
   <si>
     <t>Test ID</t>
   </si>
@@ -542,6 +542,95 @@
   <si>
     <t>Duplicate unintednded account are 
 not created.</t>
+  </si>
+  <si>
+    <t>Verify Open accounts overview</t>
+  </si>
+  <si>
+    <t>Check the open accounts overview</t>
+  </si>
+  <si>
+    <t>Account list display</t>
+  </si>
+  <si>
+    <t>Verify account numbers</t>
+  </si>
+  <si>
+    <t>Check account numbers</t>
+  </si>
+  <si>
+    <t>Correct account numbers displayed</t>
+  </si>
+  <si>
+    <t>Verify account types, Checking 
+/ Saving displayed</t>
+  </si>
+  <si>
+    <t>Check account types, Checking/
+Saving</t>
+  </si>
+  <si>
+    <t>Correct account account types displayed</t>
+  </si>
+  <si>
+    <t>Verify account balances</t>
+  </si>
+  <si>
+    <t>check account balances</t>
+  </si>
+  <si>
+    <t>Account Balance matches</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Verity open individual account</t>
+  </si>
+  <si>
+    <t>Check the individual account details</t>
+  </si>
+  <si>
+    <t>Correct accoutn details displayed</t>
+  </si>
+  <si>
+    <t>Verify newly created account</t>
+  </si>
+  <si>
+    <t>Check newly creat account</t>
+  </si>
+  <si>
+    <t>New account appears in overview</t>
+  </si>
+  <si>
+    <t>Verify account with zero balance</t>
+  </si>
+  <si>
+    <t>Check account with zero balance</t>
+  </si>
+  <si>
+    <t>Zero balance displayed correctly</t>
+  </si>
+  <si>
+    <t>Verify multiple accounts</t>
+  </si>
+  <si>
+    <t>Check multiple accounts</t>
+  </si>
+  <si>
+    <t>All user's accounts displayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High </t>
+  </si>
+  <si>
+    <t>Verify Invalid account ID</t>
+  </si>
+  <si>
+    <t>Check Invalid account ID</t>
+  </si>
+  <si>
+    <t>Invalid account isn't exposed</t>
   </si>
 </sst>
 </file>
@@ -2236,9 +2325,219 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7368FBBA-23E1-4E37-B79D-DA8AF23D4CC8}">
-  <dimension ref="A1"/>
+  <dimension ref="A4:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" t="s">
+        <v>164</v>
+      </c>
+      <c r="E5" t="s">
+        <v>165</v>
+      </c>
+      <c r="F5" t="s">
+        <v>165</v>
+      </c>
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D6" t="s">
+        <v>167</v>
+      </c>
+      <c r="E6" t="s">
+        <v>168</v>
+      </c>
+      <c r="F6" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E7" t="s">
+        <v>171</v>
+      </c>
+      <c r="F7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D8" t="s">
+        <v>173</v>
+      </c>
+      <c r="E8" t="s">
+        <v>174</v>
+      </c>
+      <c r="F8" t="s">
+        <v>174</v>
+      </c>
+      <c r="G8" t="s">
+        <v>175</v>
+      </c>
+      <c r="H8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D9" t="s">
+        <v>177</v>
+      </c>
+      <c r="E9" t="s">
+        <v>178</v>
+      </c>
+      <c r="F9" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D10" t="s">
+        <v>180</v>
+      </c>
+      <c r="E10" t="s">
+        <v>181</v>
+      </c>
+      <c r="F10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>182</v>
+      </c>
+      <c r="D11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>185</v>
+      </c>
+      <c r="D12" t="s">
+        <v>186</v>
+      </c>
+      <c r="E12" t="s">
+        <v>187</v>
+      </c>
+      <c r="F12" t="s">
+        <v>187</v>
+      </c>
+      <c r="G12" t="s">
+        <v>188</v>
+      </c>
+      <c r="H12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>189</v>
+      </c>
+      <c r="D13" t="s">
+        <v>190</v>
+      </c>
+      <c r="E13" t="s">
+        <v>191</v>
+      </c>
+      <c r="F13" t="s">
+        <v>191</v>
+      </c>
+      <c r="G13" t="s">
+        <v>175</v>
+      </c>
+      <c r="H13" t="s">
+        <v>175</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write test case for transfer funds
</commit_message>
<xml_diff>
--- a/testCases/testCases.xlsx
+++ b/testCases/testCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\projects\paraBank\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47EE7D95-E7F7-4F35-8F25-E6A9E67C8EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31E26AA-E8CC-4E5A-B40A-08ACCA1A2FC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="244">
   <si>
     <t>Test ID</t>
   </si>
@@ -631,13 +631,172 @@
   </si>
   <si>
     <t>Invalid account isn't exposed</t>
+  </si>
+  <si>
+    <t>TC_014</t>
+  </si>
+  <si>
+    <t>Verify with transfer valid amount</t>
+  </si>
+  <si>
+    <t>Check transfer valid amount</t>
+  </si>
+  <si>
+    <t>Two accounts 
+available</t>
+  </si>
+  <si>
+    <t>valid amount</t>
+  </si>
+  <si>
+    <t>Transfer successfully</t>
+  </si>
+  <si>
+    <t>Verify with transfer zero amount</t>
+  </si>
+  <si>
+    <t>Check transfer zero amount</t>
+  </si>
+  <si>
+    <t>amount - 0</t>
+  </si>
+  <si>
+    <t>Validation error</t>
+  </si>
+  <si>
+    <t>Verify with transfer negative amount</t>
+  </si>
+  <si>
+    <t>Check transfer with negative amount</t>
+  </si>
+  <si>
+    <t>Transaction reject</t>
+  </si>
+  <si>
+    <t>Verify with transfer decimal amount</t>
+  </si>
+  <si>
+    <t>Check transfer with decimal amount</t>
+  </si>
+  <si>
+    <t>Correct handling of monetary 
+value</t>
+  </si>
+  <si>
+    <t>Verify with transfer amount greater
+than balance</t>
+  </si>
+  <si>
+    <t>Check transfer with insufficient balance</t>
+  </si>
+  <si>
+    <t>insufficient amount</t>
+  </si>
+  <si>
+    <t>Transaction reject &amp; show error message</t>
+  </si>
+  <si>
+    <t>Verify same source &amp; destination</t>
+  </si>
+  <si>
+    <t>Check transfer with same source &amp; destination</t>
+  </si>
+  <si>
+    <t>select same account</t>
+  </si>
+  <si>
+    <t>Invalid transfer rejected</t>
+  </si>
+  <si>
+    <t>Verify with missing source account</t>
+  </si>
+  <si>
+    <t>Check with missing source account</t>
+  </si>
+  <si>
+    <t>Validation error display</t>
+  </si>
+  <si>
+    <t>Verify with missing destination account</t>
+  </si>
+  <si>
+    <t>Check with missing destination account</t>
+  </si>
+  <si>
+    <t>destination account blanck</t>
+  </si>
+  <si>
+    <t>source account blank</t>
+  </si>
+  <si>
+    <t>Verify with mssing amount</t>
+  </si>
+  <si>
+    <t>Check transfer with blank amount</t>
+  </si>
+  <si>
+    <t>amount  field is blank</t>
+  </si>
+  <si>
+    <t>Verify source balance</t>
+  </si>
+  <si>
+    <t>Check source balance after transfer</t>
+  </si>
+  <si>
+    <t>transfer an amount</t>
+  </si>
+  <si>
+    <t>Source balance decreases correctly</t>
+  </si>
+  <si>
+    <t>Verify destination balance</t>
+  </si>
+  <si>
+    <t>Check destination balance after transfer</t>
+  </si>
+  <si>
+    <t>Destination balance increase correctly</t>
+  </si>
+  <si>
+    <t>Verify transaction history</t>
+  </si>
+  <si>
+    <t>Check transaction history</t>
+  </si>
+  <si>
+    <t>transaction history need</t>
+  </si>
+  <si>
+    <t>View the transaction history</t>
+  </si>
+  <si>
+    <t>Verify character in amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check character in amount </t>
+  </si>
+  <si>
+    <t>abcd@#</t>
+  </si>
+  <si>
+    <t>Input rejected</t>
+  </si>
+  <si>
+    <t>Verify with very large amount</t>
+  </si>
+  <si>
+    <t>check transfer with large amount</t>
+  </si>
+  <si>
+    <t>Application handles safely</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -664,6 +823,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -682,10 +849,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -709,8 +877,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2544,9 +2715,368 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4522ED92-A484-468F-A273-7D2FF8FE5E89}">
-  <dimension ref="A1"/>
+  <dimension ref="A4:H18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="37.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D5" t="s">
+        <v>194</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="F5" t="s">
+        <v>196</v>
+      </c>
+      <c r="G5" t="s">
+        <v>197</v>
+      </c>
+      <c r="H5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D6" t="s">
+        <v>199</v>
+      </c>
+      <c r="E6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" t="s">
+        <v>200</v>
+      </c>
+      <c r="G6" t="s">
+        <v>201</v>
+      </c>
+      <c r="H6" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>202</v>
+      </c>
+      <c r="D7" t="s">
+        <v>203</v>
+      </c>
+      <c r="E7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F7">
+        <v>-100</v>
+      </c>
+      <c r="G7" t="s">
+        <v>204</v>
+      </c>
+      <c r="H7" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>205</v>
+      </c>
+      <c r="D8" t="s">
+        <v>206</v>
+      </c>
+      <c r="E8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F8">
+        <v>100.5</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" t="s">
+        <v>209</v>
+      </c>
+      <c r="E9" t="s">
+        <v>152</v>
+      </c>
+      <c r="F9" t="s">
+        <v>210</v>
+      </c>
+      <c r="G9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D10" t="s">
+        <v>213</v>
+      </c>
+      <c r="E10" t="s">
+        <v>152</v>
+      </c>
+      <c r="F10" t="s">
+        <v>214</v>
+      </c>
+      <c r="G10" t="s">
+        <v>215</v>
+      </c>
+      <c r="H10" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>216</v>
+      </c>
+      <c r="D11" t="s">
+        <v>217</v>
+      </c>
+      <c r="E11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" t="s">
+        <v>222</v>
+      </c>
+      <c r="G11" t="s">
+        <v>218</v>
+      </c>
+      <c r="H11" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>219</v>
+      </c>
+      <c r="D12" t="s">
+        <v>220</v>
+      </c>
+      <c r="E12" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" t="s">
+        <v>221</v>
+      </c>
+      <c r="G12" t="s">
+        <v>218</v>
+      </c>
+      <c r="H12" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>223</v>
+      </c>
+      <c r="D13" t="s">
+        <v>224</v>
+      </c>
+      <c r="E13" t="s">
+        <v>152</v>
+      </c>
+      <c r="F13" t="s">
+        <v>225</v>
+      </c>
+      <c r="G13" t="s">
+        <v>218</v>
+      </c>
+      <c r="H13" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>226</v>
+      </c>
+      <c r="D14" t="s">
+        <v>227</v>
+      </c>
+      <c r="E14" t="s">
+        <v>228</v>
+      </c>
+      <c r="F14">
+        <v>1000</v>
+      </c>
+      <c r="G14" t="s">
+        <v>229</v>
+      </c>
+      <c r="H14" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>230</v>
+      </c>
+      <c r="D15" t="s">
+        <v>231</v>
+      </c>
+      <c r="E15" t="s">
+        <v>228</v>
+      </c>
+      <c r="F15">
+        <v>1000</v>
+      </c>
+      <c r="G15" t="s">
+        <v>232</v>
+      </c>
+      <c r="H15" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>233</v>
+      </c>
+      <c r="D16" t="s">
+        <v>234</v>
+      </c>
+      <c r="E16" t="s">
+        <v>152</v>
+      </c>
+      <c r="F16" t="s">
+        <v>235</v>
+      </c>
+      <c r="G16" t="s">
+        <v>236</v>
+      </c>
+      <c r="H16" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>237</v>
+      </c>
+      <c r="D17" t="s">
+        <v>238</v>
+      </c>
+      <c r="E17" t="s">
+        <v>152</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="G17" t="s">
+        <v>240</v>
+      </c>
+      <c r="H17" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>192</v>
+      </c>
+      <c r="C18" t="s">
+        <v>241</v>
+      </c>
+      <c r="D18" t="s">
+        <v>242</v>
+      </c>
+      <c r="E18" t="s">
+        <v>152</v>
+      </c>
+      <c r="F18" s="10">
+        <v>999999999999</v>
+      </c>
+      <c r="G18" t="s">
+        <v>243</v>
+      </c>
+      <c r="H18" t="s">
+        <v>243</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="F17" r:id="rId1" xr:uid="{9CEFBD4D-57B5-4307-9527-DD02547ACF95}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write test case for bill payment
</commit_message>
<xml_diff>
--- a/testCases/testCases.xlsx
+++ b/testCases/testCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\projects\paraBank\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31E26AA-E8CC-4E5A-B40A-08ACCA1A2FC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB55F3D-A897-416B-8660-EC10F725A6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="294">
   <si>
     <t>Test ID</t>
   </si>
@@ -790,6 +790,156 @@
   </si>
   <si>
     <t>Application handles safely</t>
+  </si>
+  <si>
+    <t>TC_015</t>
+  </si>
+  <si>
+    <t>Verify pay bill with valid information</t>
+  </si>
+  <si>
+    <t>Check pay bill with valid information</t>
+  </si>
+  <si>
+    <t>valid information</t>
+  </si>
+  <si>
+    <t>Payment successful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priority </t>
+  </si>
+  <si>
+    <t>Criticle</t>
+  </si>
+  <si>
+    <t>Verify payee name empty</t>
+  </si>
+  <si>
+    <t>Check pay name empty</t>
+  </si>
+  <si>
+    <t>payee name blank</t>
+  </si>
+  <si>
+    <t>Validation display</t>
+  </si>
+  <si>
+    <t>Verify address empty</t>
+  </si>
+  <si>
+    <t>Check empty address field</t>
+  </si>
+  <si>
+    <t>Verify city empty</t>
+  </si>
+  <si>
+    <t>Check city empty</t>
+  </si>
+  <si>
+    <t>city empty</t>
+  </si>
+  <si>
+    <t>Verify State empty</t>
+  </si>
+  <si>
+    <t>Check state empty</t>
+  </si>
+  <si>
+    <t>Check zip empty</t>
+  </si>
+  <si>
+    <t>zip empty</t>
+  </si>
+  <si>
+    <t>Verify ZIP empty</t>
+  </si>
+  <si>
+    <t>Verify Phone empty</t>
+  </si>
+  <si>
+    <t>Check phne empty</t>
+  </si>
+  <si>
+    <t>Phone empty</t>
+  </si>
+  <si>
+    <t>Verify account number empty</t>
+  </si>
+  <si>
+    <t>Check account number empty</t>
+  </si>
+  <si>
+    <t>empty account</t>
+  </si>
+  <si>
+    <t>Verify invalid account number</t>
+  </si>
+  <si>
+    <t>Check invalid account number</t>
+  </si>
+  <si>
+    <t>invalid account</t>
+  </si>
+  <si>
+    <t>Payment rejected</t>
+  </si>
+  <si>
+    <t>Verfiy with empty acmount</t>
+  </si>
+  <si>
+    <t>check with empty amount</t>
+  </si>
+  <si>
+    <t>blank</t>
+  </si>
+  <si>
+    <t>Verify with zero amount</t>
+  </si>
+  <si>
+    <t>Check with zero amount</t>
+  </si>
+  <si>
+    <t>amount = 0</t>
+  </si>
+  <si>
+    <t>Validateion display</t>
+  </si>
+  <si>
+    <t>Verify with negative amount</t>
+  </si>
+  <si>
+    <t>Check with negative amount</t>
+  </si>
+  <si>
+    <t>Verify with insufficient balance</t>
+  </si>
+  <si>
+    <t>Check insufficient balance</t>
+  </si>
+  <si>
+    <t>Verify with decimal amount</t>
+  </si>
+  <si>
+    <t>Check with decimal amount</t>
+  </si>
+  <si>
+    <t>Correct monetary value processed</t>
+  </si>
+  <si>
+    <t>Verify payment confirmation</t>
+  </si>
+  <si>
+    <t>Check payment confirmation</t>
+  </si>
+  <si>
+    <t>Confirmation display</t>
+  </si>
+  <si>
+    <t>TC_016</t>
+  </si>
+  <si>
+    <t>Show the trasaction history</t>
   </si>
 </sst>
 </file>
@@ -2819,7 +2969,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>21</v>
       </c>
@@ -3083,9 +3233,455 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E020456B-E449-436C-B4A1-83C24244656B}">
-  <dimension ref="A1"/>
+  <dimension ref="A4:I20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>245</v>
+      </c>
+      <c r="D5" t="s">
+        <v>246</v>
+      </c>
+      <c r="E5" t="s">
+        <v>247</v>
+      </c>
+      <c r="F5" t="s">
+        <v>248</v>
+      </c>
+      <c r="G5" t="s">
+        <v>248</v>
+      </c>
+      <c r="H5" t="s">
+        <v>250</v>
+      </c>
+      <c r="I5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>251</v>
+      </c>
+      <c r="D6" t="s">
+        <v>252</v>
+      </c>
+      <c r="E6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F6" t="s">
+        <v>254</v>
+      </c>
+      <c r="G6" t="s">
+        <v>254</v>
+      </c>
+      <c r="H6" t="s">
+        <v>188</v>
+      </c>
+      <c r="I6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>255</v>
+      </c>
+      <c r="D7" t="s">
+        <v>256</v>
+      </c>
+      <c r="E7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F7" t="s">
+        <v>254</v>
+      </c>
+      <c r="G7" t="s">
+        <v>254</v>
+      </c>
+      <c r="H7" t="s">
+        <v>188</v>
+      </c>
+      <c r="I7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>257</v>
+      </c>
+      <c r="D8" t="s">
+        <v>258</v>
+      </c>
+      <c r="E8" t="s">
+        <v>259</v>
+      </c>
+      <c r="F8" t="s">
+        <v>254</v>
+      </c>
+      <c r="G8" t="s">
+        <v>254</v>
+      </c>
+      <c r="H8" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>260</v>
+      </c>
+      <c r="D9" t="s">
+        <v>261</v>
+      </c>
+      <c r="E9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F9" t="s">
+        <v>254</v>
+      </c>
+      <c r="G9" t="s">
+        <v>254</v>
+      </c>
+      <c r="H9" t="s">
+        <v>56</v>
+      </c>
+      <c r="I9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>264</v>
+      </c>
+      <c r="D10" t="s">
+        <v>262</v>
+      </c>
+      <c r="E10" t="s">
+        <v>263</v>
+      </c>
+      <c r="F10" t="s">
+        <v>254</v>
+      </c>
+      <c r="G10" t="s">
+        <v>254</v>
+      </c>
+      <c r="H10" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>265</v>
+      </c>
+      <c r="D11" t="s">
+        <v>266</v>
+      </c>
+      <c r="E11" t="s">
+        <v>267</v>
+      </c>
+      <c r="F11" t="s">
+        <v>254</v>
+      </c>
+      <c r="G11" t="s">
+        <v>254</v>
+      </c>
+      <c r="H11" t="s">
+        <v>56</v>
+      </c>
+      <c r="I11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>268</v>
+      </c>
+      <c r="D12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E12" t="s">
+        <v>270</v>
+      </c>
+      <c r="F12" t="s">
+        <v>254</v>
+      </c>
+      <c r="G12" t="s">
+        <v>254</v>
+      </c>
+      <c r="H12" t="s">
+        <v>250</v>
+      </c>
+      <c r="I12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>271</v>
+      </c>
+      <c r="D13" t="s">
+        <v>272</v>
+      </c>
+      <c r="E13" t="s">
+        <v>273</v>
+      </c>
+      <c r="F13" t="s">
+        <v>274</v>
+      </c>
+      <c r="G13" t="s">
+        <v>274</v>
+      </c>
+      <c r="H13" t="s">
+        <v>250</v>
+      </c>
+      <c r="I13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>275</v>
+      </c>
+      <c r="D14" t="s">
+        <v>276</v>
+      </c>
+      <c r="E14" t="s">
+        <v>277</v>
+      </c>
+      <c r="F14" t="s">
+        <v>254</v>
+      </c>
+      <c r="G14" t="s">
+        <v>254</v>
+      </c>
+      <c r="H14" t="s">
+        <v>250</v>
+      </c>
+      <c r="I14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>278</v>
+      </c>
+      <c r="D15" t="s">
+        <v>279</v>
+      </c>
+      <c r="E15" t="s">
+        <v>280</v>
+      </c>
+      <c r="F15" t="s">
+        <v>281</v>
+      </c>
+      <c r="G15" t="s">
+        <v>281</v>
+      </c>
+      <c r="H15" t="s">
+        <v>188</v>
+      </c>
+      <c r="I15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>282</v>
+      </c>
+      <c r="D16" t="s">
+        <v>283</v>
+      </c>
+      <c r="E16">
+        <v>-1900</v>
+      </c>
+      <c r="F16" t="s">
+        <v>281</v>
+      </c>
+      <c r="G16" t="s">
+        <v>281</v>
+      </c>
+      <c r="H16" t="s">
+        <v>188</v>
+      </c>
+      <c r="I16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>284</v>
+      </c>
+      <c r="D17" t="s">
+        <v>285</v>
+      </c>
+      <c r="E17">
+        <v>99999999</v>
+      </c>
+      <c r="F17" t="s">
+        <v>281</v>
+      </c>
+      <c r="G17" t="s">
+        <v>281</v>
+      </c>
+      <c r="H17" t="s">
+        <v>175</v>
+      </c>
+      <c r="I17" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>192</v>
+      </c>
+      <c r="C18" t="s">
+        <v>286</v>
+      </c>
+      <c r="D18" t="s">
+        <v>287</v>
+      </c>
+      <c r="E18">
+        <v>100.3</v>
+      </c>
+      <c r="F18" t="s">
+        <v>288</v>
+      </c>
+      <c r="G18" t="s">
+        <v>281</v>
+      </c>
+      <c r="H18" t="s">
+        <v>188</v>
+      </c>
+      <c r="I18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>244</v>
+      </c>
+      <c r="C19" t="s">
+        <v>289</v>
+      </c>
+      <c r="D19" t="s">
+        <v>290</v>
+      </c>
+      <c r="F19" t="s">
+        <v>291</v>
+      </c>
+      <c r="G19" t="s">
+        <v>291</v>
+      </c>
+      <c r="H19" t="s">
+        <v>188</v>
+      </c>
+      <c r="I19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>292</v>
+      </c>
+      <c r="C20" t="s">
+        <v>233</v>
+      </c>
+      <c r="D20" t="s">
+        <v>234</v>
+      </c>
+      <c r="F20" t="s">
+        <v>293</v>
+      </c>
+      <c r="G20" t="s">
+        <v>293</v>
+      </c>
+      <c r="H20" t="s">
+        <v>188</v>
+      </c>
+      <c r="I20" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write test case for find transaction history
</commit_message>
<xml_diff>
--- a/testCases/testCases.xlsx
+++ b/testCases/testCases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\projects\paraBank\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB55F3D-A897-416B-8660-EC10F725A6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C377045-B686-4323-9310-5988D8D379C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="335">
   <si>
     <t>Test ID</t>
   </si>
@@ -940,6 +940,129 @@
   </si>
   <si>
     <t>Show the trasaction history</t>
+  </si>
+  <si>
+    <t>Verify search by transaction ID</t>
+  </si>
+  <si>
+    <t>Check search by transaction ID</t>
+  </si>
+  <si>
+    <t>Valid ID</t>
+  </si>
+  <si>
+    <t>Correct transaction displayed</t>
+  </si>
+  <si>
+    <t>Verify search by amount</t>
+  </si>
+  <si>
+    <t>Check search by amount</t>
+  </si>
+  <si>
+    <t>valid transaction amount</t>
+  </si>
+  <si>
+    <t>Matching trnsactios displayed</t>
+  </si>
+  <si>
+    <t>Verify search with exact date</t>
+  </si>
+  <si>
+    <t>Check search by date</t>
+  </si>
+  <si>
+    <t>valid date</t>
+  </si>
+  <si>
+    <t>Show the matching date transaction</t>
+  </si>
+  <si>
+    <t>Matching transactios displayed</t>
+  </si>
+  <si>
+    <t>Verify search with date range</t>
+  </si>
+  <si>
+    <t>Check with date range</t>
+  </si>
+  <si>
+    <t>valid date range</t>
+  </si>
+  <si>
+    <t>Show the transaction within the date range</t>
+  </si>
+  <si>
+    <t>Verify search with month</t>
+  </si>
+  <si>
+    <t>Check search by month</t>
+  </si>
+  <si>
+    <t>Valid month</t>
+  </si>
+  <si>
+    <t>Correct monthly transactions displayed</t>
+  </si>
+  <si>
+    <t>verify search transaction type</t>
+  </si>
+  <si>
+    <t>Check search with transaction type</t>
+  </si>
+  <si>
+    <t>Credit / Debit</t>
+  </si>
+  <si>
+    <t>Selected transaction type data display</t>
+  </si>
+  <si>
+    <t>Verify search with invalid id</t>
+  </si>
+  <si>
+    <t>Check with Invalid transaction ID</t>
+  </si>
+  <si>
+    <t>Invalid transaction ID</t>
+  </si>
+  <si>
+    <t>Show the message No matchning transaction</t>
+  </si>
+  <si>
+    <t>verfiy search with blanck field</t>
+  </si>
+  <si>
+    <t>Check with blanck field</t>
+  </si>
+  <si>
+    <t>Blanck</t>
+  </si>
+  <si>
+    <t>Validation error message show.</t>
+  </si>
+  <si>
+    <t>Verify with invalid date formae</t>
+  </si>
+  <si>
+    <t>Check with Invalid date formate</t>
+  </si>
+  <si>
+    <t>invalid date</t>
+  </si>
+  <si>
+    <t>Invalid date formate</t>
+  </si>
+  <si>
+    <t>Verify with future date search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check with future date </t>
+  </si>
+  <si>
+    <t>future date</t>
+  </si>
+  <si>
+    <t>No transaction list show</t>
   </si>
 </sst>
 </file>
@@ -3688,9 +3811,307 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A65531-C65D-4E87-93C4-F541C3027ABE}">
-  <dimension ref="A1"/>
+  <dimension ref="A4:I15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" t="s">
+        <v>295</v>
+      </c>
+      <c r="E5" t="s">
+        <v>296</v>
+      </c>
+      <c r="F5" t="s">
+        <v>297</v>
+      </c>
+      <c r="G5" t="s">
+        <v>297</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>298</v>
+      </c>
+      <c r="D6" t="s">
+        <v>299</v>
+      </c>
+      <c r="E6" t="s">
+        <v>300</v>
+      </c>
+      <c r="F6" t="s">
+        <v>306</v>
+      </c>
+      <c r="G6" t="s">
+        <v>301</v>
+      </c>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>302</v>
+      </c>
+      <c r="D7" t="s">
+        <v>303</v>
+      </c>
+      <c r="E7" t="s">
+        <v>304</v>
+      </c>
+      <c r="F7" t="s">
+        <v>305</v>
+      </c>
+      <c r="G7" t="s">
+        <v>305</v>
+      </c>
+      <c r="H7" t="s">
+        <v>188</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>307</v>
+      </c>
+      <c r="D8" t="s">
+        <v>308</v>
+      </c>
+      <c r="E8" t="s">
+        <v>309</v>
+      </c>
+      <c r="F8" t="s">
+        <v>310</v>
+      </c>
+      <c r="G8" t="s">
+        <v>310</v>
+      </c>
+      <c r="H8" t="s">
+        <v>188</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>311</v>
+      </c>
+      <c r="D9" t="s">
+        <v>312</v>
+      </c>
+      <c r="E9" t="s">
+        <v>313</v>
+      </c>
+      <c r="F9" t="s">
+        <v>314</v>
+      </c>
+      <c r="G9" t="s">
+        <v>314</v>
+      </c>
+      <c r="H9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>315</v>
+      </c>
+      <c r="D10" t="s">
+        <v>316</v>
+      </c>
+      <c r="E10" t="s">
+        <v>317</v>
+      </c>
+      <c r="F10" t="s">
+        <v>318</v>
+      </c>
+      <c r="G10" t="s">
+        <v>318</v>
+      </c>
+      <c r="H10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>319</v>
+      </c>
+      <c r="D11" t="s">
+        <v>320</v>
+      </c>
+      <c r="E11" t="s">
+        <v>321</v>
+      </c>
+      <c r="F11" t="s">
+        <v>322</v>
+      </c>
+      <c r="G11" t="s">
+        <v>322</v>
+      </c>
+      <c r="H11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>323</v>
+      </c>
+      <c r="D12" t="s">
+        <v>324</v>
+      </c>
+      <c r="E12" t="s">
+        <v>325</v>
+      </c>
+      <c r="F12" t="s">
+        <v>326</v>
+      </c>
+      <c r="G12" t="s">
+        <v>326</v>
+      </c>
+      <c r="H12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>327</v>
+      </c>
+      <c r="D13" t="s">
+        <v>328</v>
+      </c>
+      <c r="E13" t="s">
+        <v>329</v>
+      </c>
+      <c r="F13" t="s">
+        <v>330</v>
+      </c>
+      <c r="G13" t="s">
+        <v>330</v>
+      </c>
+      <c r="H13" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>331</v>
+      </c>
+      <c r="D14" t="s">
+        <v>332</v>
+      </c>
+      <c r="E14" t="s">
+        <v>333</v>
+      </c>
+      <c r="F14" t="s">
+        <v>334</v>
+      </c>
+      <c r="G14" t="s">
+        <v>334</v>
+      </c>
+      <c r="H14" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>